<commit_message>
Enhancement to copy the screenshot to the shrae folder
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aci-con2\Documents\UiPath\AMP23_00_Pinturas\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0457380-F0A8-4A44-973A-036A7472BD12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{912C6C7D-5CE8-483B-A0B8-73B19D345C04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15195" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="63">
   <si>
     <t>Name</t>
   </si>
@@ -211,6 +211,9 @@
   </si>
   <si>
     <t>AMP23_00_Pinturas</t>
+  </si>
+  <si>
+    <t>PosiSoftScreenshotPath</t>
   </si>
 </sst>
 </file>
@@ -2980,7 +2983,17 @@
         <v>44</v>
       </c>
     </row>
-    <row r="6" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="6" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A6" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
     <row r="7" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="8" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="9" spans="1:26" ht="14.25" customHeight="1"/>

</xml_diff>